<commit_message>
model eval comparison file updated
</commit_message>
<xml_diff>
--- a/ML_models_pred_comparison.xlsx
+++ b/ML_models_pred_comparison.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ML Model Comparison (Class 1)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Class 1 Metrics Comparison" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -470,10 +470,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -510,7 +510,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Decision Tree Classifier</t>
+          <t>Decision Tree Classifier without Scaling</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
@@ -529,74 +529,74 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Random Forest Classifier</t>
+          <t>Random Forest Classifier without Scaling</t>
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>0.48</v>
+        <v>0.61</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>0.49</v>
+        <v>0.52</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.72</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Decision Tree Classifier with Standard Scaling</t>
+          <t>Logistic Regression without Scaling</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>0.35</v>
+        <v>0.63</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.74</v>
+        <v>0.45</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.47</v>
+        <v>0.53</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.57</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Decision Tree Classifier with MinMax Scaling</t>
+          <t>XGBoost without Scaling</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.35</v>
+        <v>0.6</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>0.74</v>
+        <v>0.51</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0.47</v>
+        <v>0.55</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.57</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Random Forest Classifier with Standard Scaling</t>
+          <t>Logistic Regression with StandardScaler</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0.61</v>
+        <v>0.62</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.52</v>
+        <v>0.53</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>0.78</v>
@@ -605,7 +605,7 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Decision Tree Classifier with Standard Scaling, SMOTEENN</t>
+          <t>Decision Tree Classifier with StandardScaler</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
@@ -624,26 +624,26 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Random Forest Classifier with Standard Scaling, SMOTEENN</t>
+          <t>Random Forest Classifier with StandardScaler</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0.35</v>
+        <v>0.61</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.74</v>
+        <v>0.45</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.47</v>
+        <v>0.52</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.57</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>XGBoost with Standard Scaling</t>
+          <t>XGBoost Classifier with StandardScaler</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
@@ -662,133 +662,304 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>XGBoost with Standard Scaling, SMOTEENN</t>
+          <t>Logistic Regression with MinMaxScaler</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>0.48</v>
+        <v>0.63</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.78</v>
+        <v>0.46</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.6</v>
+        <v>0.53</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.72</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>XGBoost with Standard Scaling, SMOTE</t>
+          <t>XGBoost with MinMaxScaler</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>0.57</v>
+        <v>0.6</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.51</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>0.57</v>
+        <v>0.55</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>XGBoost with ADASYN</t>
+          <t>Logistic Regression with StandardScaler, SMOTEENN</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0.55</v>
+        <v>0.46</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.84</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.55</v>
+        <v>0.59</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.76</v>
+        <v>0.6899999999999999</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>XGBoost with scale_pos_weight</t>
+          <t>XGBoost Classifier with StandardScaler, SMOTEENN</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>0.52</v>
+        <v>0.49</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>0.65</v>
+        <v>0.77</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Tuned XGBoost with StandardScaler and SMOTEENN</t>
+          <t>Logistic Regression with StandardScaler, SMOTE</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>0.49</v>
+        <v>0.5</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.8</v>
+        <v>0.78</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>0.61</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Tuned XGBoost with StandardScaler</t>
+          <t>XGBoost Classifier with StandardScaler, SMOTE</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>0.5</v>
+        <v>0.57</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>0.78</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>0.61</v>
+        <v>0.57</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.73</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Tuned XGBoost with StandardScaler and Optuna</t>
+          <t>Logistic Regression with StandardScaler, ADASYN</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>0.49</v>
+        <v>0.48</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>0.61</v>
       </c>
       <c r="E16" s="3" t="n">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>XGBoost Classifier with StandardScaler, ADASYN</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>XGBoost with scale_pos_weight</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Cost-Sensitive AdaBoost</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Logistic Regression with StandardScaler and Class Weights</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Tuned Logistic Regression with StandardScaler and SMOTE</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Tuned XGBoost (No Scaling, No SMOTEENN)</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Tuned XGBoost with StandardScaler</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Tuned XGBoost with StandardScaler and SMOTEENN</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Tuned XGBoost with StandardScaler and Optuna</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="E25" s="5" t="n">
         <v>0.73</v>
       </c>
     </row>

</xml_diff>